<commit_message>
Initial steps to create spatial data.
</commit_message>
<xml_diff>
--- a/output_tables/group_summary_old.xlsx
+++ b/output_tables/group_summary_old.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/output_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="94" documentId="8_{59E47FFB-B8F7-45C3-A319-0743BC9995C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{997CAE2A-F15E-4B14-8716-7C65909F7ED7}"/>
+  <xr:revisionPtr revIDLastSave="98" documentId="8_{59E47FFB-B8F7-45C3-A319-0743BC9995C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AC35531-8A54-4CEE-8F04-3D3E3C8254D6}"/>
   <bookViews>
-    <workbookView xWindow="15" yWindow="90" windowWidth="28785" windowHeight="15390" xr2:uid="{DE4F24FA-FBA3-478C-9F9E-E001BBB69A88}"/>
+    <workbookView xWindow="0" yWindow="90" windowWidth="26505" windowHeight="15390" xr2:uid="{DE4F24FA-FBA3-478C-9F9E-E001BBB69A88}"/>
   </bookViews>
   <sheets>
     <sheet name="group_summary" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="236">
   <si>
     <t>group_no</t>
   </si>
@@ -761,6 +761,9 @@
   </si>
   <si>
     <t>donor_site_code</t>
+  </si>
+  <si>
+    <t>Others</t>
   </si>
 </sst>
 </file>
@@ -1351,6 +1354,1081 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="7"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="8"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="9"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="10"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="11"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="12"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="13"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="14"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>group_summary!$P$12:$P$26</c:f>
+              <c:strCache>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>DuPont Wharf</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Rocky Bay</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Dumas Bay</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Thompson Cove</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Windy Bluff</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Point Julia</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Quilcene Bay</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Sandy Point</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Anderson Island</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Creosote Point</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Cutts Island</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Skagit Bay</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Ketron Island</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Henry Island</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Others</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>group_summary!$Q$12:$Q$26</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3778-4E1C-8DEB-8B979A4DDBC5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>329405</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>41275</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>444499</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>174625</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93E67C62-3228-F72F-6739-84DC82FCDC39}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="DOWTY, PETER (DNR)" id="{750E6FC1-6785-B14C-B0F3-55122449730F}" userId="S::peter.dowty@dnr.wa.gov::01cf875a-4e15-4928-8f93-7a0dfa1efb6b" providerId="AD"/>
@@ -1682,7 +2760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A4FED8F-716B-4B06-A141-CFC261A1ADE2}">
-  <dimension ref="A1:M196"/>
+  <dimension ref="A1:Q196"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1698,7 +2776,7 @@
     <col min="19" max="19" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1712,7 +2790,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1729,7 +2807,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1746,7 +2824,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1769,7 +2847,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1795,7 +2873,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1828,7 +2906,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1854,7 +2932,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1887,7 +2965,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1917,7 +2995,7 @@
         <v>5.128205128205128E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1943,7 +3021,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1969,7 +3047,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1994,8 +3072,14 @@
       <c r="K12" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P12" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q12">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2020,8 +3104,14 @@
       <c r="K13" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P13" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q13">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2046,8 +3136,14 @@
       <c r="K14" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P14" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q14">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2072,8 +3168,14 @@
       <c r="K15" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P15" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q15">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2098,8 +3200,14 @@
       <c r="K16" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P16" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q16">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2124,8 +3232,14 @@
       <c r="K17" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P17" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q17">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2150,8 +3264,14 @@
       <c r="K18" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P18" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q18">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2176,8 +3296,14 @@
       <c r="K19" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P19" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q19">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2202,8 +3328,14 @@
       <c r="K20" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P20" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q20">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2228,8 +3360,14 @@
       <c r="K21" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P21" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q21">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2254,8 +3392,14 @@
       <c r="K22" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q22">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2283,8 +3427,14 @@
       <c r="K23" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P23" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q23">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2309,8 +3459,14 @@
       <c r="K24" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P24" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2335,8 +3491,14 @@
       <c r="K25" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P25" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2361,8 +3523,15 @@
       <c r="K26" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="P26" t="s">
+        <v>235</v>
+      </c>
+      <c r="Q26">
+        <f>SUM(J19:J27)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2388,7 +3557,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2414,7 +3583,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2437,7 +3606,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2460,7 +3629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2483,7 +3652,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -5326,7 +6495,8 @@
     <sortCondition ref="R5:R29"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>